<commit_message>
adding demo of movable table
</commit_message>
<xml_diff>
--- a/data/info.xlsx
+++ b/data/info.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28224"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeaeduco-my.sharepoint.com/personal/nelson_parra_udea_edu_co/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D095A395-C9AA-4810-B2EA-6B2175CC550E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{D095A395-C9AA-4810-B2EA-6B2175CC550E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD0AA042-425C-43F1-82E1-63B685D99FAA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{081945B4-ACDB-4922-979C-0964006EAE99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -56,118 +56,118 @@
     <t>Lorem Ipsum 1</t>
   </si>
   <si>
+    <t xml:space="preserve">LM14-16 </t>
+  </si>
+  <si>
+    <t>Dolor sit amet 1</t>
+  </si>
+  <si>
+    <t>dsa1@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 2</t>
   </si>
   <si>
+    <t>W8-11</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 2</t>
+  </si>
+  <si>
+    <t>dsa2@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 3</t>
   </si>
   <si>
+    <t>J6-8 M6-8</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 3</t>
+  </si>
+  <si>
+    <t>dsa3@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 4</t>
   </si>
   <si>
+    <t>LM14-17</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 4</t>
+  </si>
+  <si>
+    <t>dsa4@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 5</t>
   </si>
   <si>
+    <t>W8-12</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 5</t>
+  </si>
+  <si>
+    <t>dsa5@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 6</t>
   </si>
   <si>
+    <t>J6-8 M8-7</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 6</t>
+  </si>
+  <si>
+    <t>dsa6@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 7</t>
   </si>
   <si>
+    <t>LM14-18</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 7</t>
+  </si>
+  <si>
+    <t>dsa7@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 8</t>
   </si>
   <si>
+    <t>W8-13</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 8</t>
+  </si>
+  <si>
+    <t>dsa8@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 9</t>
   </si>
   <si>
+    <t>J6-8 M10-12</t>
+  </si>
+  <si>
+    <t>Dolor sit amet 9</t>
+  </si>
+  <si>
+    <t>dsa9@udea</t>
+  </si>
+  <si>
     <t>Lorem Ipsum 10</t>
   </si>
   <si>
-    <t xml:space="preserve">LM14-16 </t>
-  </si>
-  <si>
-    <t>W8-11</t>
-  </si>
-  <si>
-    <t>J6-8 M8-6</t>
-  </si>
-  <si>
-    <t>LM14-17</t>
-  </si>
-  <si>
-    <t>W8-12</t>
-  </si>
-  <si>
-    <t>J6-8 M8-7</t>
-  </si>
-  <si>
-    <t>LM14-18</t>
-  </si>
-  <si>
-    <t>W8-13</t>
-  </si>
-  <si>
-    <t>J6-8 M8-8</t>
-  </si>
-  <si>
     <t>LM14-19</t>
   </si>
   <si>
-    <t>Dolor sit amet 1</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 2</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 3</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 4</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 5</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 6</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 7</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 8</t>
-  </si>
-  <si>
-    <t>Dolor sit amet 9</t>
-  </si>
-  <si>
     <t>Dolor sit amet 10</t>
-  </si>
-  <si>
-    <t>dsa1@udea</t>
-  </si>
-  <si>
-    <t>dsa2@udea</t>
-  </si>
-  <si>
-    <t>dsa3@udea</t>
-  </si>
-  <si>
-    <t>dsa4@udea</t>
-  </si>
-  <si>
-    <t>dsa5@udea</t>
-  </si>
-  <si>
-    <t>dsa6@udea</t>
-  </si>
-  <si>
-    <t>dsa7@udea</t>
-  </si>
-  <si>
-    <t>dsa8@udea</t>
-  </si>
-  <si>
-    <t>dsa9@udea</t>
   </si>
   <si>
     <t>dsa10@udea</t>
@@ -177,7 +177,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -560,15 +560,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F911FDE0-43DE-4028-8474-08261371C8D5}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="13.90625" customWidth="1"/>
-    <col min="3" max="3" width="16.36328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -585,7 +585,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -593,163 +593,163 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>44</v>

</xml_diff>